<commit_message>
feat: implement core management modules and administrative UI for user, module, and training program oversight
</commit_message>
<xml_diff>
--- a/Aplikasi PD Rev01.xlsx
+++ b/Aplikasi PD Rev01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Kerjaan Pengembangan dan Mutu\7. Project\Aplikasi PDQA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\mycode\ihatec-modul\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82872081-DE95-4E42-9F73-2AE9F64360A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{928C5FAC-7AF6-43CD-A9DD-E8420AB6B5DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="5" activeTab="8" xr2:uid="{B1353187-EE38-4CDA-9616-D23759397E26}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" firstSheet="2" activeTab="4" xr2:uid="{B1353187-EE38-4CDA-9616-D23759397E26}"/>
   </bookViews>
   <sheets>
     <sheet name="General Flow" sheetId="1" r:id="rId1"/>
@@ -1246,7 +1246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1295,6 +1295,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1304,34 +1310,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1342,14 +1343,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3404,8 +3401,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2400307" y="3318720"/>
-          <a:ext cx="1085845" cy="148387"/>
+          <a:off x="2291722" y="3334912"/>
+          <a:ext cx="1085845" cy="150292"/>
           <a:chOff x="5996423" y="2895653"/>
           <a:chExt cx="943454" cy="160284"/>
         </a:xfrm>
@@ -3604,8 +3601,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="5857875" y="4953001"/>
-          <a:ext cx="1085845" cy="148387"/>
+          <a:off x="5596890" y="4986338"/>
+          <a:ext cx="1062985" cy="150292"/>
           <a:chOff x="5996423" y="2895653"/>
           <a:chExt cx="943454" cy="160284"/>
         </a:xfrm>
@@ -3848,8 +3845,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="5186362" y="6367464"/>
-          <a:ext cx="1085845" cy="166686"/>
+          <a:off x="4963477" y="6416041"/>
+          <a:ext cx="1047745" cy="168591"/>
           <a:chOff x="5996423" y="2895653"/>
           <a:chExt cx="943454" cy="160284"/>
         </a:xfrm>
@@ -4048,8 +4045,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2395538" y="10367964"/>
-          <a:ext cx="1085845" cy="148387"/>
+          <a:off x="2286953" y="10458451"/>
+          <a:ext cx="1085845" cy="150292"/>
           <a:chOff x="5996423" y="2895653"/>
           <a:chExt cx="943454" cy="160284"/>
         </a:xfrm>
@@ -4248,8 +4245,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2395538" y="12358689"/>
-          <a:ext cx="1085845" cy="148387"/>
+          <a:off x="2286953" y="12470131"/>
+          <a:ext cx="1085845" cy="150292"/>
           <a:chOff x="5996423" y="2895653"/>
           <a:chExt cx="943454" cy="160284"/>
         </a:xfrm>
@@ -4448,8 +4445,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2395538" y="14168439"/>
-          <a:ext cx="1085845" cy="148387"/>
+          <a:off x="2286953" y="14298931"/>
+          <a:ext cx="1085845" cy="150292"/>
           <a:chOff x="5996423" y="2895653"/>
           <a:chExt cx="943454" cy="160284"/>
         </a:xfrm>
@@ -4648,8 +4645,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2395538" y="15616239"/>
-          <a:ext cx="1085845" cy="148387"/>
+          <a:off x="2286953" y="15761971"/>
+          <a:ext cx="1085845" cy="150292"/>
           <a:chOff x="5996423" y="2895653"/>
           <a:chExt cx="943454" cy="160284"/>
         </a:xfrm>
@@ -4848,8 +4845,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2395538" y="17245014"/>
-          <a:ext cx="1085845" cy="148387"/>
+          <a:off x="2286953" y="17407891"/>
+          <a:ext cx="1085845" cy="150292"/>
           <a:chOff x="5996423" y="2895653"/>
           <a:chExt cx="943454" cy="160284"/>
         </a:xfrm>
@@ -5048,8 +5045,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2395538" y="18692814"/>
-          <a:ext cx="1085845" cy="148387"/>
+          <a:off x="2286953" y="18870931"/>
+          <a:ext cx="1085845" cy="150292"/>
           <a:chOff x="5996423" y="2895653"/>
           <a:chExt cx="943454" cy="160284"/>
         </a:xfrm>
@@ -5248,8 +5245,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2395538" y="8920164"/>
-          <a:ext cx="1085845" cy="148387"/>
+          <a:off x="2286953" y="8995411"/>
+          <a:ext cx="1085845" cy="150292"/>
           <a:chOff x="5996423" y="2895653"/>
           <a:chExt cx="943454" cy="160284"/>
         </a:xfrm>
@@ -5448,8 +5445,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="5186362" y="7634289"/>
-          <a:ext cx="1085845" cy="148387"/>
+          <a:off x="4963477" y="7696201"/>
+          <a:ext cx="1047745" cy="150292"/>
           <a:chOff x="5996423" y="2895653"/>
           <a:chExt cx="943454" cy="160284"/>
         </a:xfrm>
@@ -9515,9 +9512,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{151E1552-8AE1-485C-ABC3-BB8C0074F188}">
   <dimension ref="D2"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="4:4" ht="34.15" x14ac:dyDescent="1.05">
+    <row r="2" spans="4:4" ht="33.6" x14ac:dyDescent="0.65">
       <c r="D2" s="1" t="s">
         <v>34</v>
       </c>
@@ -9531,14 +9528,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B92C7DC8-E675-4E13-AD0A-EB163AF145B5}">
   <dimension ref="A2:E104"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.59765625" customWidth="1"/>
-    <col min="3" max="3" width="39.46484375" customWidth="1"/>
-    <col min="5" max="5" width="9.06640625" customWidth="1"/>
+    <col min="2" max="2" width="23.5546875" customWidth="1"/>
+    <col min="3" max="3" width="39.44140625" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -9546,7 +9543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>2</v>
       </c>
@@ -9554,7 +9551,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>7</v>
       </c>
@@ -9562,7 +9559,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>4</v>
       </c>
@@ -9570,7 +9567,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>9</v>
       </c>
@@ -9578,7 +9575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>6</v>
       </c>
@@ -9586,12 +9583,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
@@ -9602,7 +9599,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1</v>
       </c>
@@ -9610,7 +9607,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2</v>
       </c>
@@ -9618,7 +9615,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>3</v>
       </c>
@@ -9626,12 +9623,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -9648,7 +9645,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -9656,7 +9653,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>24</v>
       </c>
@@ -9670,37 +9667,37 @@
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:4" s="38" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="37" t="s">
+    <row r="37" spans="1:4" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="30" t="s">
         <v>192</v>
       </c>
-      <c r="C37" s="37" t="s">
+      <c r="C37" s="30" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="38" spans="1:4" s="38" customFormat="1" x14ac:dyDescent="0.45"/>
-    <row r="39" spans="1:4" s="38" customFormat="1" x14ac:dyDescent="0.45"/>
-    <row r="40" spans="1:4" s="38" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="37" t="s">
+    <row r="38" spans="1:4" s="31" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="1:4" s="31" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="1:4" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="B40" s="37" t="s">
+      <c r="B40" s="30" t="s">
         <v>193</v>
       </c>
-      <c r="C40" s="37" t="s">
+      <c r="C40" s="30" t="s">
         <v>191</v>
       </c>
-      <c r="D40" s="37" t="s">
+      <c r="D40" s="30" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="41" spans="1:4" s="38" customFormat="1" x14ac:dyDescent="0.45"/>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:4" s="31" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="13" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>24</v>
       </c>
@@ -9711,22 +9708,22 @@
         <v>17</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="13" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>24</v>
       </c>
@@ -9737,37 +9734,37 @@
         <v>17</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>24</v>
       </c>
@@ -9778,33 +9775,33 @@
         <v>17</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" s="2"/>
       <c r="B70" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>24</v>
       </c>
@@ -9815,25 +9812,25 @@
         <v>17</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="2"/>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>24</v>
       </c>
@@ -9844,27 +9841,27 @@
         <v>17</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>24</v>
       </c>
@@ -9875,22 +9872,22 @@
         <v>17</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>24</v>
       </c>
@@ -9901,17 +9898,17 @@
         <v>17</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>179</v>
       </c>
@@ -9925,24 +9922,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90854903-8ABC-4B8E-941E-1317E6E242A4}">
   <dimension ref="G9:V29"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="9" width="18.73046875" customWidth="1"/>
-    <col min="10" max="11" width="15.46484375" customWidth="1"/>
-    <col min="12" max="12" width="13.59765625" customWidth="1"/>
-    <col min="13" max="13" width="12.3984375" customWidth="1"/>
-    <col min="14" max="14" width="13.796875" customWidth="1"/>
-    <col min="15" max="15" width="18.3984375" customWidth="1"/>
+    <col min="8" max="9" width="18.77734375" customWidth="1"/>
+    <col min="10" max="11" width="15.44140625" customWidth="1"/>
+    <col min="12" max="12" width="13.5546875" customWidth="1"/>
+    <col min="13" max="13" width="12.44140625" customWidth="1"/>
+    <col min="14" max="14" width="13.77734375" customWidth="1"/>
+    <col min="15" max="15" width="18.44140625" customWidth="1"/>
     <col min="16" max="16" width="20.6640625" customWidth="1"/>
-    <col min="17" max="17" width="17.19921875" customWidth="1"/>
-    <col min="18" max="18" width="19.19921875" customWidth="1"/>
+    <col min="17" max="17" width="17.21875" customWidth="1"/>
+    <col min="18" max="18" width="19.21875" customWidth="1"/>
     <col min="19" max="19" width="23.6640625" customWidth="1"/>
-    <col min="20" max="20" width="17.1328125" customWidth="1"/>
+    <col min="20" max="20" width="17.109375" customWidth="1"/>
     <col min="21" max="21" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="7:22" x14ac:dyDescent="0.45">
+    <row r="9" spans="7:22" x14ac:dyDescent="0.3">
       <c r="N9" s="4" t="s">
         <v>11</v>
       </c>
@@ -9965,7 +9962,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="7:22" x14ac:dyDescent="0.45">
+    <row r="10" spans="7:22" x14ac:dyDescent="0.3">
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -9976,7 +9973,7 @@
       </c>
       <c r="T10" s="3"/>
     </row>
-    <row r="11" spans="7:22" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="7:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -9987,7 +9984,7 @@
       </c>
       <c r="T11" s="3"/>
     </row>
-    <row r="12" spans="7:22" x14ac:dyDescent="0.45">
+    <row r="12" spans="7:22" x14ac:dyDescent="0.3">
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -9996,7 +9993,7 @@
       <c r="S12" s="3"/>
       <c r="T12" s="3"/>
     </row>
-    <row r="16" spans="7:22" x14ac:dyDescent="0.45">
+    <row r="16" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G16" s="18" t="s">
         <v>11</v>
       </c>
@@ -10027,16 +10024,16 @@
       <c r="P16" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="Q16" s="51" t="s">
+      <c r="Q16" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="R16" s="51" t="s">
+      <c r="R16" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="S16" s="51" t="s">
+      <c r="S16" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="T16" s="51" t="s">
+      <c r="T16" s="18" t="s">
         <v>210</v>
       </c>
       <c r="U16" s="18" t="s">
@@ -10046,19 +10043,19 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="7:22" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="17" spans="7:22" ht="43.2" x14ac:dyDescent="0.3">
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
-      <c r="J17" s="41" t="s">
+      <c r="J17" s="37" t="s">
         <v>194</v>
       </c>
-      <c r="K17" s="42"/>
+      <c r="K17" s="38"/>
       <c r="L17" s="39" t="s">
         <v>195</v>
       </c>
-      <c r="M17" s="43"/>
-      <c r="N17" s="40"/>
+      <c r="M17" s="40"/>
+      <c r="N17" s="41"/>
       <c r="O17" s="3"/>
       <c r="P17" s="14" t="s">
         <v>209</v>
@@ -10066,7 +10063,7 @@
       <c r="Q17" s="3"/>
       <c r="R17" s="3"/>
       <c r="S17" s="3"/>
-      <c r="T17" s="52" t="s">
+      <c r="T17" s="33" t="s">
         <v>207</v>
       </c>
       <c r="U17" s="23" t="s">
@@ -10074,7 +10071,7 @@
       </c>
       <c r="V17" s="3"/>
     </row>
-    <row r="18" spans="7:22" x14ac:dyDescent="0.45">
+    <row r="18" spans="7:22" x14ac:dyDescent="0.3">
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -10092,7 +10089,7 @@
       <c r="U18" s="3"/>
       <c r="V18" s="3"/>
     </row>
-    <row r="29" spans="7:22" x14ac:dyDescent="0.45">
+    <row r="29" spans="7:22" x14ac:dyDescent="0.3">
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
     </row>
@@ -10109,24 +10106,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E33A1FA9-A269-4C0E-87A4-BC8FC01301B5}">
   <dimension ref="A2:XFD36"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.9296875" customWidth="1"/>
-    <col min="2" max="2" width="1.796875" customWidth="1"/>
+    <col min="1" max="1" width="27.88671875" customWidth="1"/>
+    <col min="2" max="2" width="1.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9 16384:16384" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:9 16384:16384" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>31</v>
       </c>
       <c r="XFD2" s="2"/>
     </row>
-    <row r="6" spans="1:9 16384:16384" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:9 16384:16384" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:9 16384:16384" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:9 16384:16384" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>45</v>
       </c>
@@ -10134,7 +10131,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:9 16384:16384" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:9 16384:16384" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>49</v>
       </c>
@@ -10142,7 +10139,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:9 16384:16384" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:9 16384:16384" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>46</v>
       </c>
@@ -10150,7 +10147,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:9 16384:16384" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:9 16384:16384" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -10158,7 +10155,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:9 16384:16384" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:9 16384:16384" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>51</v>
       </c>
@@ -10166,7 +10163,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:9 16384:16384" s="8" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:9 16384:16384" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>58</v>
       </c>
@@ -10174,7 +10171,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:9 16384:16384" s="8" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:9 16384:16384" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>64</v>
       </c>
@@ -10182,7 +10179,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:9 16384:16384" s="8" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:9 16384:16384" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>59</v>
       </c>
@@ -10197,7 +10194,7 @@
       <c r="H15" s="10"/>
       <c r="I15" s="10"/>
     </row>
-    <row r="16" spans="1:9 16384:16384" s="8" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:9 16384:16384" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>62</v>
       </c>
@@ -10205,7 +10202,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>63</v>
       </c>
@@ -10213,7 +10210,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>65</v>
       </c>
@@ -10221,7 +10218,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>60</v>
       </c>
@@ -10232,7 +10229,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>61</v>
       </c>
@@ -10240,17 +10237,17 @@
         <v>73</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -10258,7 +10255,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>68</v>
       </c>
@@ -10266,7 +10263,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>69</v>
       </c>
@@ -10274,7 +10271,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>66</v>
       </c>
@@ -10282,7 +10279,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>81</v>
       </c>
@@ -10291,22 +10288,22 @@
         <v>82</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="15" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>93</v>
       </c>
@@ -10320,32 +10317,32 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B25801B-F65D-4848-8AEE-26F75E9B66B6}">
   <dimension ref="A2:K55"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.59765625" customWidth="1"/>
-    <col min="2" max="2" width="1.796875" customWidth="1"/>
-    <col min="3" max="3" width="21.73046875" customWidth="1"/>
-    <col min="4" max="4" width="22.19921875" customWidth="1"/>
-    <col min="5" max="5" width="23.265625" customWidth="1"/>
-    <col min="6" max="6" width="21.265625" customWidth="1"/>
+    <col min="1" max="1" width="32.5546875" customWidth="1"/>
+    <col min="2" max="2" width="1.77734375" customWidth="1"/>
+    <col min="3" max="3" width="85.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.21875" customWidth="1"/>
+    <col min="5" max="5" width="23.21875" customWidth="1"/>
+    <col min="6" max="6" width="21.21875" customWidth="1"/>
     <col min="7" max="7" width="19" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
     <col min="9" max="9" width="26" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="14.19921875" customWidth="1"/>
+    <col min="11" max="11" width="14.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>45</v>
       </c>
@@ -10357,7 +10354,7 @@
       </c>
       <c r="D8" s="7"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>86</v>
       </c>
@@ -10369,7 +10366,7 @@
       </c>
       <c r="D9" s="7"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>189</v>
       </c>
@@ -10381,7 +10378,7 @@
       </c>
       <c r="D10" s="7"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>199</v>
       </c>
@@ -10393,7 +10390,7 @@
       </c>
       <c r="D11" s="7"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>95</v>
       </c>
@@ -10405,7 +10402,7 @@
       </c>
       <c r="D12" s="7"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>65</v>
       </c>
@@ -10417,7 +10414,7 @@
       </c>
       <c r="D13" s="7"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>60</v>
       </c>
@@ -10429,7 +10426,7 @@
       </c>
       <c r="D14" s="7"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -10441,7 +10438,7 @@
       </c>
       <c r="D15" s="7"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>51</v>
       </c>
@@ -10453,8 +10450,8 @@
       </c>
       <c r="D16" s="7"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A17" s="37" t="s">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="30" t="s">
         <v>118</v>
       </c>
       <c r="B17" t="s">
@@ -10465,7 +10462,7 @@
       </c>
       <c r="D17" s="7"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C18" s="18" t="s">
         <v>99</v>
       </c>
@@ -10494,11 +10491,11 @@
         <v>67</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="63.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="33" t="s">
+    <row r="19" spans="1:11" ht="63.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="43" t="s">
         <v>105</v>
       </c>
-      <c r="B19" s="33"/>
+      <c r="B19" s="43"/>
       <c r="C19" s="19" t="s">
         <v>36</v>
       </c>
@@ -10517,7 +10514,7 @@
       <c r="H19" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="I19" s="34" t="s">
+      <c r="I19" s="44" t="s">
         <v>104</v>
       </c>
       <c r="J19" s="19" t="s">
@@ -10527,9 +10524,9 @@
         <v>107</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A20" s="33"/>
-      <c r="B20" s="33"/>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="43"/>
+      <c r="B20" s="43"/>
       <c r="C20" s="19" t="s">
         <v>37</v>
       </c>
@@ -10548,7 +10545,7 @@
       <c r="H20" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="I20" s="34"/>
+      <c r="I20" s="44"/>
       <c r="J20" s="19" t="s">
         <v>132</v>
       </c>
@@ -10556,9 +10553,9 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A21" s="33"/>
-      <c r="B21" s="33"/>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="43"/>
+      <c r="B21" s="43"/>
       <c r="C21" s="19" t="s">
         <v>38</v>
       </c>
@@ -10577,7 +10574,7 @@
       <c r="H21" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="I21" s="34"/>
+      <c r="I21" s="44"/>
       <c r="J21" s="19" t="s">
         <v>132</v>
       </c>
@@ -10585,8 +10582,8 @@
         <v>107</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A23" s="37" t="s">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="30" t="s">
         <v>197</v>
       </c>
       <c r="B23" t="s">
@@ -10595,7 +10592,7 @@
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C24" s="18" t="s">
         <v>193</v>
       </c>
@@ -10621,9 +10618,9 @@
         <v>202</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="63.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="33"/>
-      <c r="B25" s="33"/>
+    <row r="25" spans="1:11" ht="63.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="43"/>
+      <c r="B25" s="43"/>
       <c r="C25" s="14" t="s">
         <v>200</v>
       </c>
@@ -10639,7 +10636,7 @@
       <c r="G25" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H25" s="44" t="s">
+      <c r="H25" s="45" t="s">
         <v>201</v>
       </c>
       <c r="I25" s="19" t="s">
@@ -10649,9 +10646,9 @@
         <v>107</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A26" s="33"/>
-      <c r="B26" s="33"/>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" s="43"/>
+      <c r="B26" s="43"/>
       <c r="C26" s="19" t="s">
         <v>70</v>
       </c>
@@ -10667,7 +10664,7 @@
       <c r="G26" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H26" s="45"/>
+      <c r="H26" s="46"/>
       <c r="I26" s="19" t="s">
         <v>132</v>
       </c>
@@ -10675,9 +10672,9 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="33"/>
-      <c r="B27" s="33"/>
+    <row r="27" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="43"/>
+      <c r="B27" s="43"/>
       <c r="C27" s="19" t="s">
         <v>70</v>
       </c>
@@ -10693,7 +10690,7 @@
       <c r="G27" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H27" s="46"/>
+      <c r="H27" s="47"/>
       <c r="I27" s="19" t="s">
         <v>132</v>
       </c>
@@ -10701,12 +10698,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>45</v>
       </c>
@@ -10720,7 +10717,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>86</v>
       </c>
@@ -10734,7 +10731,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>88</v>
       </c>
@@ -10748,7 +10745,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>95</v>
       </c>
@@ -10762,7 +10759,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>65</v>
       </c>
@@ -10777,7 +10774,7 @@
       </c>
       <c r="E38" s="7"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>96</v>
       </c>
@@ -10791,7 +10788,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>51</v>
       </c>
@@ -10805,12 +10802,12 @@
         <v>53</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C42" s="18" t="s">
         <v>40</v>
       </c>
@@ -10839,9 +10836,9 @@
         <v>67</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="63.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A43" s="33"/>
-      <c r="B43" s="33"/>
+    <row r="43" spans="1:11" ht="63.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="43"/>
+      <c r="B43" s="43"/>
       <c r="C43" s="19" t="s">
         <v>36</v>
       </c>
@@ -10870,9 +10867,9 @@
         <v>126</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A44" s="33"/>
-      <c r="B44" s="33"/>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="43"/>
+      <c r="B44" s="43"/>
       <c r="C44" s="19" t="s">
         <v>37</v>
       </c>
@@ -10901,9 +10898,9 @@
         <v>126</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A45" s="33"/>
-      <c r="B45" s="33"/>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="43"/>
+      <c r="B45" s="43"/>
       <c r="C45" s="19" t="s">
         <v>38</v>
       </c>
@@ -10932,50 +10929,50 @@
         <v>126</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" s="17"/>
       <c r="B46" s="17"/>
-      <c r="C46" s="47"/>
-      <c r="D46" s="48"/>
-      <c r="E46" s="48"/>
-      <c r="F46" s="48"/>
-      <c r="G46" s="48"/>
-      <c r="H46" s="48"/>
-      <c r="I46" s="49"/>
-      <c r="J46" s="48"/>
-      <c r="K46" s="48"/>
-    </row>
-    <row r="47" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" s="50" t="s">
+      <c r="C46" s="7"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="20"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="20"/>
+      <c r="H46" s="20"/>
+      <c r="I46" s="32"/>
+      <c r="J46" s="20"/>
+      <c r="K46" s="20"/>
+    </row>
+    <row r="47" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="42" t="s">
         <v>203</v>
       </c>
-      <c r="B47" s="50"/>
-      <c r="C47" s="50"/>
-      <c r="D47" s="50"/>
-      <c r="E47" s="50"/>
-      <c r="F47" s="48"/>
-      <c r="G47" s="48"/>
-      <c r="H47" s="48"/>
-      <c r="I47" s="49"/>
-      <c r="J47" s="48"/>
-      <c r="K47" s="48"/>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B47" s="42"/>
+      <c r="C47" s="42"/>
+      <c r="D47" s="42"/>
+      <c r="E47" s="42"/>
+      <c r="F47" s="20"/>
+      <c r="G47" s="20"/>
+      <c r="H47" s="20"/>
+      <c r="I47" s="32"/>
+      <c r="J47" s="20"/>
+      <c r="K47" s="20"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="54" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A54" s="10" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="55" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A55" s="10" t="s">
         <v>204</v>
       </c>
@@ -10999,29 +10996,29 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0517BA89-D325-4E48-9929-0B1A1642B4D0}">
   <dimension ref="A3:H8"/>
-  <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.06640625" style="6"/>
-    <col min="2" max="3" width="18.19921875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="21.86328125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="20.53125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="6"/>
+    <col min="2" max="3" width="18.21875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="21.88671875" style="6" customWidth="1"/>
+    <col min="5" max="5" width="20.5546875" style="6" customWidth="1"/>
     <col min="6" max="6" width="21.33203125" style="6" customWidth="1"/>
     <col min="7" max="7" width="18.6640625" style="6" customWidth="1"/>
-    <col min="8" max="8" width="13.06640625" style="6" customWidth="1"/>
-    <col min="9" max="16384" width="9.06640625" style="6"/>
+    <col min="8" max="8" width="13.109375" style="6" customWidth="1"/>
+    <col min="9" max="16384" width="9.109375" style="6"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E4" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>24</v>
       </c>
@@ -11047,14 +11044,14 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="38.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="B8" s="35" t="s">
+    <row r="8" spans="1:8" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="48" t="s">
         <v>136</v>
       </c>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11069,29 +11066,29 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{746E0441-8C20-45B2-BC89-6778493205AF}">
   <dimension ref="A3:G8"/>
-  <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.06640625" style="6"/>
-    <col min="2" max="2" width="18.19921875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="21.86328125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="20.53125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="6"/>
+    <col min="2" max="2" width="18.21875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="21.88671875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="20.5546875" style="6" customWidth="1"/>
     <col min="5" max="5" width="21.33203125" style="6" customWidth="1"/>
     <col min="6" max="6" width="18.6640625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="13.06640625" style="6" customWidth="1"/>
-    <col min="8" max="16384" width="9.06640625" style="6"/>
+    <col min="7" max="7" width="13.109375" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="9.109375" style="6"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D4" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>24</v>
       </c>
@@ -11114,11 +11111,11 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="B8" s="35"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
+    <row r="8" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11133,25 +11130,25 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4AE8AD1-FABB-464C-BBD8-CFF1C886DCE8}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.19921875" customWidth="1"/>
+    <col min="1" max="1" width="14.21875" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="14.53125" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
     <col min="4" max="4" width="22.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -11159,7 +11156,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>143</v>
       </c>
@@ -11173,24 +11170,24 @@
         <v>103</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B9" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="C9" s="36" t="s">
+      <c r="C9" s="49" t="s">
         <v>146</v>
       </c>
-      <c r="D9" s="36"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D9" s="49"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
@@ -11198,7 +11195,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>143</v>
       </c>
@@ -11212,7 +11209,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>149</v>
       </c>
@@ -11223,7 +11220,7 @@
         <v>46199</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>150</v>
       </c>
@@ -11234,7 +11231,7 @@
         <v>46199</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>129</v>
       </c>
@@ -11257,46 +11254,46 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{239D5422-757A-4FF7-B93E-B6A0CC7ACD16}">
   <dimension ref="A2:L13"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.06640625" style="16"/>
-    <col min="2" max="2" width="28.06640625" style="16" customWidth="1"/>
-    <col min="3" max="3" width="24.3984375" style="16" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="16"/>
+    <col min="2" max="2" width="28.109375" style="16" customWidth="1"/>
+    <col min="3" max="3" width="24.44140625" style="16" customWidth="1"/>
     <col min="4" max="4" width="20.33203125" style="16" customWidth="1"/>
     <col min="5" max="5" width="23" style="16" customWidth="1"/>
-    <col min="6" max="6" width="27.06640625" style="16" customWidth="1"/>
-    <col min="7" max="7" width="28.06640625" style="16" customWidth="1"/>
-    <col min="8" max="8" width="21.3984375" style="16" customWidth="1"/>
-    <col min="9" max="9" width="24.06640625" style="16" customWidth="1"/>
-    <col min="10" max="10" width="26.86328125" style="16" customWidth="1"/>
-    <col min="11" max="11" width="27.9296875" style="16" customWidth="1"/>
-    <col min="12" max="12" width="16.06640625" style="16" customWidth="1"/>
-    <col min="13" max="16384" width="9.06640625" style="16"/>
+    <col min="6" max="6" width="27.109375" style="16" customWidth="1"/>
+    <col min="7" max="7" width="28.109375" style="16" customWidth="1"/>
+    <col min="8" max="8" width="21.44140625" style="16" customWidth="1"/>
+    <col min="9" max="9" width="24.109375" style="16" customWidth="1"/>
+    <col min="10" max="10" width="26.88671875" style="16" customWidth="1"/>
+    <col min="11" max="11" width="27.88671875" style="16" customWidth="1"/>
+    <col min="12" max="12" width="16.109375" style="16" customWidth="1"/>
+    <col min="13" max="16384" width="9.109375" style="16"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:12" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="31" t="s">
+    <row r="2" spans="1:12" ht="17.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-    </row>
-    <row r="3" spans="1:12" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+    </row>
+    <row r="3" spans="1:12" ht="17.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="29"/>
       <c r="B3" s="29"/>
       <c r="C3" s="29"/>
       <c r="D3" s="29"/>
     </row>
-    <row r="4" spans="1:12" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="31" t="s">
+    <row r="4" spans="1:12" ht="17.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="35" t="s">
         <v>185</v>
       </c>
-      <c r="B4" s="31"/>
+      <c r="B4" s="35"/>
       <c r="C4" s="29"/>
       <c r="D4" s="29"/>
     </row>
-    <row r="7" spans="1:12" s="28" customFormat="1" ht="26.25" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:12" s="28" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
         <v>152</v>
       </c>
@@ -11334,11 +11331,11 @@
         <v>184</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A8" s="30" t="s">
+    <row r="8" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="34" t="s">
         <v>147</v>
       </c>
-      <c r="B8" s="30"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="16" t="s">
         <v>163</v>
       </c>
@@ -11367,12 +11364,12 @@
         <v>183</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="32" t="s">
+    <row r="13" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="36" t="s">
         <v>186</v>
       </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>